<commit_message>
feat: evolve universal bank schema from source evidence
</commit_message>
<xml_diff>
--- a/template/Bank_CDKT_ReportNormId.v2.xlsx
+++ b/template/Bank_CDKT_ReportNormId.v2.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
   <si>
     <t>ReportNormId</t>
   </si>
@@ -259,6 +259,63 @@
   </si>
   <si>
     <t>TỔNG VỐN CHỦ SỞ HỮU</t>
+  </si>
+  <si>
+    <t>Dự phòng rủi ro chứng khoán kinh doanh</t>
+  </si>
+  <si>
+    <t>Dự phòng rủi ro chứng khoán đầu tư</t>
+  </si>
+  <si>
+    <t>Tiền gửi và vay Chính phủ, NHNN</t>
+  </si>
+  <si>
+    <t>CHỈ TIÊU NGOÀI BÁO CÁO TÌNH HÌNH TÀI CHÍNH HỢP NHẤT</t>
+  </si>
+  <si>
+    <t>Nghĩa vụ nợ tiềm ẩn</t>
+  </si>
+  <si>
+    <t>Bảo lãnh vay vốn</t>
+  </si>
+  <si>
+    <t>Cam kết giao dịch hối đoái</t>
+  </si>
+  <si>
+    <t>- Cam kết mua ngoại tệ</t>
+  </si>
+  <si>
+    <t>- Cam kết bán ngoại tệ</t>
+  </si>
+  <si>
+    <t>- Cam kết nhận - giao dịch hoán đổi tiền tệ</t>
+  </si>
+  <si>
+    <t>- Cam kết trả - giao dịch hoán đổi tiền tệ</t>
+  </si>
+  <si>
+    <t>Cam kết trong nghiệp vụ L/C</t>
+  </si>
+  <si>
+    <t>Bảo lãnh khác</t>
+  </si>
+  <si>
+    <t>Các cam kết khác</t>
+  </si>
+  <si>
+    <t>Trong đó: hạn mức tín dụng chưa sử dụng có thể hủy ngang</t>
+  </si>
+  <si>
+    <t>Các khoản mục ngoại bảng khác</t>
+  </si>
+  <si>
+    <t>Lãi cho vay và phí phải thu chưa thu được</t>
+  </si>
+  <si>
+    <t>Nợ khó đòi đã xử lý</t>
+  </si>
+  <si>
+    <t>Tài sản và chứng từ khác</t>
   </si>
 </sst>
 </file>
@@ -626,7 +683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
@@ -745,10 +802,10 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>4347</v>
+        <v>6035</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -756,10 +813,10 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>4314</v>
+        <v>4347</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -767,10 +824,10 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>4315</v>
+        <v>4314</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -778,10 +835,10 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>4348</v>
+        <v>4315</v>
       </c>
       <c r="C14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -789,10 +846,10 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>4349</v>
+        <v>4348</v>
       </c>
       <c r="C15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -800,10 +857,10 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>5322</v>
+        <v>4349</v>
       </c>
       <c r="C16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -811,10 +868,10 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>5323</v>
+        <v>5322</v>
       </c>
       <c r="C17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -822,10 +879,10 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>5324</v>
+        <v>5323</v>
       </c>
       <c r="C18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -833,10 +890,10 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>4316</v>
+        <v>5324</v>
       </c>
       <c r="C19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -844,10 +901,10 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>4350</v>
+        <v>4316</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -855,10 +912,10 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>4351</v>
+        <v>4350</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -866,10 +923,10 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>4352</v>
+        <v>4351</v>
       </c>
       <c r="C22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -877,10 +934,10 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>4317</v>
+        <v>6036</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -888,10 +945,10 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>4333</v>
+        <v>4352</v>
       </c>
       <c r="C24" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -899,10 +956,10 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>4354</v>
+        <v>4317</v>
       </c>
       <c r="C25" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -910,10 +967,10 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>4334</v>
+        <v>4333</v>
       </c>
       <c r="C26" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -921,10 +978,10 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>4355</v>
+        <v>4354</v>
       </c>
       <c r="C27" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -932,10 +989,10 @@
         <v>26</v>
       </c>
       <c r="B28">
-        <v>4307</v>
+        <v>4334</v>
       </c>
       <c r="C28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -943,10 +1000,10 @@
         <v>27</v>
       </c>
       <c r="B29">
-        <v>4328</v>
+        <v>4355</v>
       </c>
       <c r="C29" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -954,10 +1011,10 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>4367</v>
+        <v>4307</v>
       </c>
       <c r="C30" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -965,10 +1022,10 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>4368</v>
+        <v>4328</v>
       </c>
       <c r="C31" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -976,10 +1033,10 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>4329</v>
+        <v>4367</v>
       </c>
       <c r="C32" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -987,10 +1044,10 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>4369</v>
+        <v>4368</v>
       </c>
       <c r="C33" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -998,10 +1055,10 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>4370</v>
+        <v>4329</v>
       </c>
       <c r="C34" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1009,10 +1066,10 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>4330</v>
+        <v>4369</v>
       </c>
       <c r="C35" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1020,10 +1077,10 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>4371</v>
+        <v>4370</v>
       </c>
       <c r="C36" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1031,10 +1088,10 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>4372</v>
+        <v>4330</v>
       </c>
       <c r="C37" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1042,10 +1099,10 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>4308</v>
+        <v>4371</v>
       </c>
       <c r="C38" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1053,10 +1110,10 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>4331</v>
+        <v>4372</v>
       </c>
       <c r="C39" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1064,10 +1121,10 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>4332</v>
+        <v>4308</v>
       </c>
       <c r="C40" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1075,10 +1132,10 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>4327</v>
+        <v>4331</v>
       </c>
       <c r="C41" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1086,10 +1143,10 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>4356</v>
+        <v>4332</v>
       </c>
       <c r="C42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1097,10 +1154,10 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>4357</v>
+        <v>4327</v>
       </c>
       <c r="C43" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1108,10 +1165,10 @@
         <v>42</v>
       </c>
       <c r="B44">
-        <v>4335</v>
+        <v>4356</v>
       </c>
       <c r="C44" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1119,10 +1176,10 @@
         <v>43</v>
       </c>
       <c r="B45">
-        <v>4366</v>
+        <v>4357</v>
       </c>
       <c r="C45" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1130,10 +1187,10 @@
         <v>44</v>
       </c>
       <c r="B46">
-        <v>4309</v>
+        <v>4335</v>
       </c>
       <c r="C46" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1141,10 +1198,10 @@
         <v>45</v>
       </c>
       <c r="B47">
-        <v>4358</v>
+        <v>4366</v>
       </c>
       <c r="C47" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1152,10 +1209,10 @@
         <v>46</v>
       </c>
       <c r="B48">
-        <v>4375</v>
+        <v>4309</v>
       </c>
       <c r="C48" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1163,10 +1220,10 @@
         <v>47</v>
       </c>
       <c r="B49">
-        <v>4303</v>
+        <v>4358</v>
       </c>
       <c r="C49" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1174,10 +1231,10 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>4318</v>
+        <v>4375</v>
       </c>
       <c r="C50" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1185,10 +1242,10 @@
         <v>49</v>
       </c>
       <c r="B51">
-        <v>4319</v>
+        <v>4303</v>
       </c>
       <c r="C51" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1196,10 +1253,10 @@
         <v>50</v>
       </c>
       <c r="B52">
-        <v>4359</v>
+        <v>4318</v>
       </c>
       <c r="C52" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1207,10 +1264,10 @@
         <v>51</v>
       </c>
       <c r="B53">
-        <v>4360</v>
+        <v>6037</v>
       </c>
       <c r="C53" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1218,10 +1275,10 @@
         <v>52</v>
       </c>
       <c r="B54">
-        <v>4320</v>
+        <v>4319</v>
       </c>
       <c r="C54" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1229,10 +1286,10 @@
         <v>53</v>
       </c>
       <c r="B55">
-        <v>4321</v>
+        <v>4359</v>
       </c>
       <c r="C55" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1240,10 +1297,10 @@
         <v>54</v>
       </c>
       <c r="B56">
-        <v>4322</v>
+        <v>4360</v>
       </c>
       <c r="C56" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1251,10 +1308,10 @@
         <v>55</v>
       </c>
       <c r="B57">
-        <v>4323</v>
+        <v>4320</v>
       </c>
       <c r="C57" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1262,10 +1319,10 @@
         <v>56</v>
       </c>
       <c r="B58">
-        <v>4324</v>
+        <v>4321</v>
       </c>
       <c r="C58" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1273,10 +1330,10 @@
         <v>57</v>
       </c>
       <c r="B59">
-        <v>4361</v>
+        <v>4322</v>
       </c>
       <c r="C59" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1284,10 +1341,10 @@
         <v>58</v>
       </c>
       <c r="B60">
-        <v>4336</v>
+        <v>4323</v>
       </c>
       <c r="C60" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1295,10 +1352,10 @@
         <v>59</v>
       </c>
       <c r="B61">
-        <v>4362</v>
+        <v>4324</v>
       </c>
       <c r="C61" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1306,10 +1363,10 @@
         <v>60</v>
       </c>
       <c r="B62">
-        <v>4363</v>
+        <v>4361</v>
       </c>
       <c r="C62" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1317,10 +1374,10 @@
         <v>61</v>
       </c>
       <c r="B63">
-        <v>4304</v>
+        <v>4336</v>
       </c>
       <c r="C63" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1328,10 +1385,10 @@
         <v>62</v>
       </c>
       <c r="B64">
-        <v>4325</v>
+        <v>4362</v>
       </c>
       <c r="C64" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1339,10 +1396,10 @@
         <v>63</v>
       </c>
       <c r="B65">
-        <v>4364</v>
+        <v>4363</v>
       </c>
       <c r="C65" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1350,10 +1407,10 @@
         <v>64</v>
       </c>
       <c r="B66">
-        <v>4337</v>
+        <v>4304</v>
       </c>
       <c r="C66" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1361,10 +1418,10 @@
         <v>65</v>
       </c>
       <c r="B67">
-        <v>4373</v>
+        <v>4325</v>
       </c>
       <c r="C67" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1372,10 +1429,10 @@
         <v>66</v>
       </c>
       <c r="B68">
-        <v>4338</v>
+        <v>4364</v>
       </c>
       <c r="C68" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1383,10 +1440,10 @@
         <v>67</v>
       </c>
       <c r="B69">
-        <v>4340</v>
+        <v>4337</v>
       </c>
       <c r="C69" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1394,10 +1451,10 @@
         <v>68</v>
       </c>
       <c r="B70">
-        <v>4374</v>
+        <v>4373</v>
       </c>
       <c r="C70" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1405,10 +1462,10 @@
         <v>69</v>
       </c>
       <c r="B71">
-        <v>4339</v>
+        <v>4338</v>
       </c>
       <c r="C71" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1416,10 +1473,10 @@
         <v>70</v>
       </c>
       <c r="B72">
-        <v>4365</v>
+        <v>4340</v>
       </c>
       <c r="C72" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1427,10 +1484,10 @@
         <v>71</v>
       </c>
       <c r="B73">
-        <v>4342</v>
+        <v>4374</v>
       </c>
       <c r="C73" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1438,10 +1495,10 @@
         <v>72</v>
       </c>
       <c r="B74">
-        <v>4341</v>
+        <v>4339</v>
       </c>
       <c r="C74" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1449,10 +1506,10 @@
         <v>73</v>
       </c>
       <c r="B75">
-        <v>4343</v>
+        <v>4365</v>
       </c>
       <c r="C75" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1460,10 +1517,10 @@
         <v>74</v>
       </c>
       <c r="B76">
-        <v>5699</v>
+        <v>4342</v>
       </c>
       <c r="C76" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1471,10 +1528,10 @@
         <v>75</v>
       </c>
       <c r="B77">
-        <v>4306</v>
+        <v>4341</v>
       </c>
       <c r="C77" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1482,10 +1539,10 @@
         <v>76</v>
       </c>
       <c r="B78">
-        <v>5712</v>
+        <v>4343</v>
       </c>
       <c r="C78" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="15" x14ac:dyDescent="0.2">
@@ -1493,10 +1550,219 @@
         <v>77</v>
       </c>
       <c r="B79">
+        <v>5699</v>
+      </c>
+      <c r="C79" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A80" s="1">
+        <v>78</v>
+      </c>
+      <c r="B80">
+        <v>4306</v>
+      </c>
+      <c r="C80" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A81" s="1">
+        <v>79</v>
+      </c>
+      <c r="B81">
+        <v>5712</v>
+      </c>
+      <c r="C81" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A82" s="1">
+        <v>80</v>
+      </c>
+      <c r="B82">
         <v>4305</v>
       </c>
-      <c r="C79" t="s">
+      <c r="C82" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A83" s="1">
+        <v>81</v>
+      </c>
+      <c r="B83">
+        <v>6038</v>
+      </c>
+      <c r="C83" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A84" s="1">
+        <v>82</v>
+      </c>
+      <c r="B84">
+        <v>6039</v>
+      </c>
+      <c r="C84" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A85" s="1">
+        <v>83</v>
+      </c>
+      <c r="B85">
+        <v>6040</v>
+      </c>
+      <c r="C85" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A86" s="1">
+        <v>84</v>
+      </c>
+      <c r="B86">
+        <v>6041</v>
+      </c>
+      <c r="C86" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A87" s="1">
+        <v>85</v>
+      </c>
+      <c r="B87">
+        <v>6042</v>
+      </c>
+      <c r="C87" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A88" s="1">
+        <v>86</v>
+      </c>
+      <c r="B88">
+        <v>6043</v>
+      </c>
+      <c r="C88" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A89" s="1">
+        <v>87</v>
+      </c>
+      <c r="B89">
+        <v>6044</v>
+      </c>
+      <c r="C89" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A90" s="1">
+        <v>88</v>
+      </c>
+      <c r="B90">
+        <v>6045</v>
+      </c>
+      <c r="C90" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A91" s="1">
+        <v>89</v>
+      </c>
+      <c r="B91">
+        <v>6046</v>
+      </c>
+      <c r="C91" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A92" s="1">
+        <v>90</v>
+      </c>
+      <c r="B92">
+        <v>6047</v>
+      </c>
+      <c r="C92" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A93" s="1">
+        <v>91</v>
+      </c>
+      <c r="B93">
+        <v>6048</v>
+      </c>
+      <c r="C93" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A94" s="1">
+        <v>92</v>
+      </c>
+      <c r="B94">
+        <v>6049</v>
+      </c>
+      <c r="C94" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A95" s="1">
+        <v>93</v>
+      </c>
+      <c r="B95">
+        <v>6050</v>
+      </c>
+      <c r="C95" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A96" s="1">
+        <v>94</v>
+      </c>
+      <c r="B96">
+        <v>6051</v>
+      </c>
+      <c r="C96" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A97" s="1">
+        <v>95</v>
+      </c>
+      <c r="B97">
+        <v>6052</v>
+      </c>
+      <c r="C97" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A98" s="1">
+        <v>96</v>
+      </c>
+      <c r="B98">
+        <v>6053</v>
+      </c>
+      <c r="C98" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>